<commit_message>
improve: use plain audit commentary and concrete review guidance
</commit_message>
<xml_diff>
--- a/docs/evidence/business_report_preview.xlsx
+++ b/docs/evidence/business_report_preview.xlsx
@@ -888,7 +888,7 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Stored risk classifications identify records to prioritize for human review; they are not adjudicated audit outcomes.</t>
+          <t>Risk scores help reviewers decide which transactions to check first. A high score alone does not establish wrongdoing.</t>
         </is>
       </c>
     </row>
@@ -900,11 +900,11 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Prioritization can direct review effort toward records with stronger stored risk indicators while retaining attention to incomplete assessments.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="40" customHeight="1">
+          <t>Reviewing higher-risk records first may help the team focus its work. Lower-risk and unscored records can still need review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="48" customHeight="1">
       <c r="A27" s="3" t="inlineStr">
         <is>
           <t>III. F1 — Recommended Review (BASELINE)</t>
@@ -912,7 +912,7 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Inspect the linked transaction and rule evidence, obtain supporting documents and record the investigation outcome.</t>
+          <t>Start with the linked higher-risk transactions and inspect their failed-rule evidence. Request the relevant invoices and approval records, compare them with the flagged issue and record the review outcome.</t>
         </is>
       </c>
     </row>
@@ -952,7 +952,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="40" customHeight="1">
+    <row r="31" ht="48" customHeight="1">
       <c r="A31" s="3" t="inlineStr">
         <is>
           <t>III. F2 — Recommended Review (BASELINE)</t>
@@ -960,7 +960,7 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Reconcile supplier onboarding and registry records and inspect supporting invoices before deciding whether the vendor relationship is valid.</t>
+          <t>Compare the vendor registration used by the rule with supplier onboarding records. Request supporting invoices and record whether the supplier relationship can be verified.</t>
         </is>
       </c>
     </row>
@@ -1000,7 +1000,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="40" customHeight="1">
+    <row r="35" ht="48" customHeight="1">
       <c r="A35" s="3" t="inlineStr">
         <is>
           <t>III. F3 — Recommended Review (BASELINE)</t>
@@ -1008,7 +1008,7 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Confirm assignment, review notes and case decisions and check that any proposed remediation has supporting evidence.</t>
+          <t>For any listed alerts or cases, check the assigned reviewer, review notes and closure evidence. Record outstanding work separately from completed checks.</t>
         </is>
       </c>
     </row>
@@ -1032,7 +1032,7 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>Transaction-level evaluation does not establish that every configured rule had sufficient input and context to execute.</t>
+          <t>A transaction may have passed through an executed rule while other checks could not run.</t>
         </is>
       </c>
     </row>
@@ -1044,11 +1044,11 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Unavailable fields or context can limit the conclusions that management can draw from automated checks.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="40" customHeight="1">
+          <t>Missing inputs can leave gaps in the checks and limit the conclusions drawn from the report.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="48" customHeight="1">
       <c r="A39" s="3" t="inlineStr">
         <is>
           <t>III. F4 — Recommended Review (BASELINE)</t>
@@ -1056,7 +1056,7 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>Inspect per-rule coverage and exclusion reasons and reconcile missing inputs with the responsible data owner.</t>
+          <t>Use the rule-coverage appendix to identify checks that did not run and their missing inputs. Ask the data owner to reconcile those inputs and record the remaining gaps.</t>
         </is>
       </c>
     </row>
@@ -1224,7 +1224,7 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>business-findings-1.0.0</t>
+          <t>business-findings-1.0.2</t>
         </is>
       </c>
     </row>

</xml_diff>